<commit_message>
case: clean STL filenames; docs: prettier BOM.xlsx (sections/zebra) + white PETG & Bambu Lab 3mf notes
</commit_message>
<xml_diff>
--- a/docs/MSXnano_BOM.xlsx
+++ b/docs/MSXnano_BOM.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,14 +30,33 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="007F6000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -46,7 +65,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="002F5496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F6FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,13 +115,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -449,282 +507,309 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>MSXnano — Piezas de la carcasa (impresión 3D)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>🖨  Imprime todo con  case/msxnano_case_bambulab.3mf  (proyecto Bambu Lab).   Material recomendado: PETG BLANCO.</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Pieza</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Fichero</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Link (descarga/origen)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Superior izquierda</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Upper_Left.stl.stl</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>upper_left.stl</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="6" t="inlineStr"/>
+      <c r="F4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Superior derecha</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Upper_Right.stl.stl</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>upper_right.stl</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="8" t="inlineStr"/>
+      <c r="F5" s="8" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Inferior izquierda</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Lower left.stl</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>lower_left.stl</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="6" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Inferior derecha</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Lower_Right.stl</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>lower_right.stl</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="8" t="inlineStr"/>
+      <c r="F7" s="8" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Lateral inferior (TN20K v4)</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>tn20k_case_v4-lower_side.stl</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Lateral inferior</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>lower_side.stl</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="6" t="inlineStr"/>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>TN20K case v4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Soporte teclado A</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Keyboard_Support.stl_A.stl</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>keyboard_support_a.stl</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="8" t="inlineStr"/>
+      <c r="F9" s="8" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Soporte teclado B</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Keyboard_Support.stl_B.stl</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>keyboard_support_b.stl</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="6" t="inlineStr"/>
+      <c r="F10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Soporte placa</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Raspberry_Support.stl.stl</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Soporte de placa</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>raspberry_support.stl</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="8" t="inlineStr"/>
+      <c r="F11" s="8" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Pilar 1</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Pillar1_x2.stl.stl</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="n">
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>pillar1.stl</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>imprimir x2</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="E12" s="6" t="inlineStr"/>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>imprimir ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Pilar 2</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Pillar2_x2.stl.stl</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="n">
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>pillar2.stl</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>imprimir x2</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="E13" s="8" t="inlineStr"/>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>imprimir ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Proyecto completo (3MF)</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>MINIMSX.3mf</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>archivo 3MF con todas las piezas</t>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Proyecto Bambu Lab (todo)</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>msxnano_case_bambulab.3mf</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="6" t="inlineStr"/>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>abre en Bambu Studio e imprime todo de una</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -735,253 +820,311 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>MSXnano — Lista de componentes (BOM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Componente</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Link (compra)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Núcleo</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Sipeed Tang Nano 20K (FPGA GW2AR-18)</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Placa principal; BL616 USB-HID y 6 LEDs onboard</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="C4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="6" t="inlineStr"/>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Placa principal · BL616 USB-HID y 6 LEDs onboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Tarjeta microSD</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Imagenes de disco / Nextor (FAT)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="C5" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="8" t="inlineStr"/>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Imágenes de disco / Nextor (FAT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Cable USB-C</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Alimentacion + programacion (Gowin)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="C6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="6" t="inlineStr"/>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Alimentación + programación (Gowin)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Cable HDMI</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Salida de video</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="C7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="8" t="inlineStr"/>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Salida de vídeo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Teclado USB (USB-A)</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="C8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="6" t="inlineStr"/>
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>Al puerto USB-A host del BL616</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>Mando (opcional)</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n"/>
+      <c r="C9" s="3" t="n"/>
+      <c r="D9" s="3" t="n"/>
+      <c r="E9" s="3" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Hub USB (opcional)</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Solo para teclado + mando a la vez</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Hub USB</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="8" t="inlineStr"/>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Sólo para teclado + mando a la vez</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Mando USB (opcional)</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Mando USB</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="6" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>XInput/Xbox recomendado</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>WiFi (opcional)</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Modulo ESP-01S (ESP8266) (opcional)</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>WiFi/UNAPI. TX-&gt;77, RX-&gt;73, VCC-&gt;3.3V, GND-&gt;GND</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>Módulo ESP-01S (ESP8266)</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="8" t="inlineStr"/>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>TX→pin 77, RX→pin 73, VCC→3.3V, GND→GND · firmware ducasp ESPFW1.4 (OCM)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Cables/jumpers para ESP (opcional)</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Conexion al header</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Cables / jumpers para ESP</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="6" t="inlineStr"/>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Conexión al header GPIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>Carcasa</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Carcasa impresa en 3D</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Ver hoja "Piezas 3D (case)"</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Carcasa impresa en 3D (PETG blanco)</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="8" t="inlineStr"/>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>STL/3MF en case/ · ver hoja "Piezas 3D (case)"</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Tornilleria / separadores</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Segun carcasa (rellenar)</t>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Tornillería / separadores</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="6" t="inlineStr"/>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>según carcasa (rellenar)</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(BOM): add purchase links (AliExpress) + fix typos (Micro, USB-C)
</commit_message>
<xml_diff>
--- a/docs/MSXnano_BOM.xlsx
+++ b/docs/MSXnano_BOM.xlsx
@@ -2,23 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28905" yWindow="0" windowWidth="28815" windowHeight="15585" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Piezas 3D (case)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Componentes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,31 +28,39 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="007F6000"/>
+      <color rgb="FF7F6000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00000000"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="FF1F3864"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -65,31 +72,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="FF1F3864"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F5496"/>
+        <fgColor rgb="FF2F5496"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F6FC"/>
+        <fgColor rgb="FFF2F6FC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
+        <fgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -99,31 +106,70 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -139,12 +185,26 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -508,298 +568,298 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="5" customWidth="1" style="9" min="1" max="1"/>
+    <col width="26" customWidth="1" style="9" min="2" max="2"/>
+    <col width="30" customWidth="1" style="9" min="3" max="3"/>
+    <col width="10" customWidth="1" style="9" min="4" max="4"/>
+    <col width="38" customWidth="1" style="9" min="5" max="5"/>
+    <col width="34" customWidth="1" style="9" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="26" customHeight="1" s="9">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>MSXnano — Piezas de la carcasa (impresión 3D)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="2" ht="22" customHeight="1" s="9">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>🖨  Imprime todo con  case/msxnano_case_bambulab.3mf  (proyecto Bambu Lab).   Material recomendado: PETG BLANCO.</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="B2" s="12" t="n"/>
+      <c r="C2" s="12" t="n"/>
+      <c r="D2" s="12" t="n"/>
+      <c r="E2" s="12" t="n"/>
+      <c r="F2" s="13" t="n"/>
+    </row>
+    <row r="3" ht="20" customHeight="1" s="9">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Pieza</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Fichero</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>Link (descarga/origen)</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Superior izquierda</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>upper_left.stl</t>
         </is>
       </c>
-      <c r="D4" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
+      <c r="D4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="3" t="n"/>
+      <c r="F4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="n">
+      <c r="A5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Superior derecha</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>upper_right.stl</t>
         </is>
       </c>
-      <c r="D5" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="8" t="inlineStr"/>
-      <c r="F5" s="8" t="inlineStr"/>
+      <c r="D5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Inferior izquierda</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>lower_left.stl</t>
         </is>
       </c>
-      <c r="D6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
+      <c r="D6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="3" t="n"/>
+      <c r="F6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Inferior derecha</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>lower_right.stl</t>
         </is>
       </c>
-      <c r="D7" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="8" t="inlineStr"/>
-      <c r="F7" s="8" t="inlineStr"/>
+      <c r="D7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Lateral inferior</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>lower_side.stl</t>
         </is>
       </c>
-      <c r="D8" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="6" t="inlineStr"/>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="D8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="3" t="n"/>
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>TN20K case v4</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Soporte teclado A</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>keyboard_support_a.stl</t>
         </is>
       </c>
-      <c r="D9" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="8" t="inlineStr"/>
-      <c r="F9" s="8" t="inlineStr"/>
+      <c r="D9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Soporte teclado B</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>keyboard_support_b.stl</t>
         </is>
       </c>
-      <c r="D10" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="6" t="inlineStr"/>
-      <c r="F10" s="6" t="inlineStr"/>
+      <c r="D10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="3" t="n"/>
+      <c r="F10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Soporte de placa</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>raspberry_support.stl</t>
         </is>
       </c>
-      <c r="D11" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="8" t="inlineStr"/>
-      <c r="F11" s="8" t="inlineStr"/>
+      <c r="D11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n">
+      <c r="A12" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Pilar 1</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>pillar1.stl</t>
         </is>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D12" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="6" t="inlineStr"/>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>imprimir ×2</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="n">
+      <c r="A13" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Pilar 2</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>pillar2.stl</t>
         </is>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="8" t="inlineStr"/>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>imprimir ×2</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="n">
+    <row r="14" ht="28" customHeight="1" s="9">
+      <c r="A14" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Proyecto Bambu Lab (todo)</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>msxnano_case_bambulab.3mf</t>
         </is>
       </c>
-      <c r="D14" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="6" t="inlineStr"/>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="D14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="3" t="n"/>
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>abre en Bambu Studio e imprime todo de una</t>
         </is>
@@ -820,311 +880,282 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" style="9" min="1" max="1"/>
+    <col width="40" customWidth="1" style="9" min="2" max="2"/>
+    <col width="10" customWidth="1" style="9" min="3" max="3"/>
+    <col width="85.6328125" customWidth="1" style="9" min="4" max="4"/>
+    <col width="46" customWidth="1" style="9" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="26" customHeight="1" s="9">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>MSXnano — Lista de componentes (BOM)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
+    <row r="2" ht="20" customHeight="1" s="9">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>Componente</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>Link (compra)</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Núcleo</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B3" s="12" t="n"/>
+      <c r="C3" s="12" t="n"/>
+      <c r="D3" s="12" t="n"/>
+      <c r="E3" s="13" t="n"/>
+    </row>
+    <row r="4" ht="29" customHeight="1" s="9">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Sipeed Tang Nano 20K (FPGA GW2AR-18)</t>
         </is>
       </c>
-      <c r="C4" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="C4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>https://es.aliexpress.com/item/1005005581148230.html?spm=a2g0o.store_pc_home.promoteWysiwyg_6000843307735.1005005581148230&amp;gatewayAdapt=glo2esp</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Placa principal · BL616 USB-HID y 6 LEDs onboard</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="n">
+    <row r="5" ht="182" customHeight="1" s="9">
+      <c r="A5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>Tarjeta microSD</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="8" t="inlineStr"/>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Conector Hembra MicroSD a Micro SD 15cm</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>https://es.aliexpress.com/item/1005004124859525.html?gps-id=pcStoreLeaderboard&amp;scm=1007.22922.271278.0&amp;scm_id=1007.22922.271278.0&amp;scm-url=1007.22922.271278.0&amp;pvid=1dcd5058-de05-4451-b9a1-40ef94365aad&amp;_t=gps-id%3ApcStoreLeaderboard%2Cscm-url%3A1007.22922.271278.0%2Cpvid%3A1dcd5058-de05-4451-b9a1-40ef94365aad%2Ctpp_buckets%3A668%232846%238109%231935&amp;pdp_ext_f=%7B%22order%22%3A%221230%22%2C%22eval%22%3A%221%22%2C%22sceneId%22%3A%2212922%22%2C%22fromPage%22%3A%22recommend%22%7D&amp;pdp_npi=6%40dis%21EUR%213.04%212.79%21%21%213.46%213.18%21%402103973d17802464014145440e1291%2112000028118186957%21rec%21ES%21129485342%21XZ%211%210%21n_tag%3A-29919%3Bd%3A90000c2b%3Bm03_new_user%3A-29895&amp;spm=a2g0o.store_pc_home.smartLeaderboard_971065810.1005004124859525&amp;gatewayAdapt=glo2esp</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Imágenes de disco / Nextor (FAT)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Cable USB-C</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Cable USB-C internos 20cm</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>https://es.aliexpress.com/item/1005006806265814.html?gps-id=pcStoreJustForYou&amp;scm=1007.23125.137358.0&amp;scm_id=1007.23125.137358.0&amp;scm-url=1007.23125.137358.0&amp;pvid=0a0eccd2-bf03-449f-902d-4bee2d7162cd&amp;_t=gps-id%3ApcStoreJustForYou%2Cscm-url%3A1007.23125.137358.0%2Cpvid%3A0a0eccd2-bf03-449f-902d-4bee2d7162cd%2Ctpp_buckets%3A668%232846%238109%231935&amp;pdp_ext_f=%7B%22order%22%3A%22329%22%2C%22eval%22%3A%221%22%2C%22sceneId%22%3A%2213125%22%2C%22fromPage%22%3A%22recommend%22%7D&amp;pdp_npi=6%40dis%21EUR%212.17%212.17%21%21%212.47%212.47%21%402103973d17802463232242634e1291%2112000038369249748%21rec%21ES%21129485342%21X%211%210%21n_tag%3A-29919%3Bd%3A90000c2b%3Bm03_new_user%3A-29895&amp;spm=a2g0o.store_pc_home.smartJustForYou_2004001802241.1005006806265814&amp;gatewayAdapt=glo2esp</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Alimentación + programación (Gowin)</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
+    <row r="7" ht="28" customHeight="1" s="9">
+      <c r="A7" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>Cable HDMI</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="8" t="inlineStr"/>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Conector Hembra USB-C</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>https://es.aliexpress.com/item/1005003355262263.html?spm=a2g0o.order_list.order_list_main.756.413d194dwWlj7h&amp;gatewayAdapt=glo2esp</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Salida de vídeo</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Conector HDMI Hembra</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n"/>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>https://es.aliexpress.com/item/1005001975924049.html?spm=a2g0o.order_list.order_list_main.745.413d194dwWlj7h&amp;gatewayAdapt=glo2esp</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="n"/>
+    </row>
+    <row r="9" ht="28" customHeight="1" s="9">
+      <c r="A9" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Conector Hembra HDMI 15cm</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>https://es.aliexpress.com/item/1005009220802088.html?spm=a2g0o.order_list.order_list_main.35.413d194dwWlj7h&amp;gatewayAdapt=glo2esp</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Al puerto USB-A host del BL616</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Teclado USB (USB-A)</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="6" t="inlineStr"/>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="C10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Ajazz AK33</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Al puerto USB-A host del BL616</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>Mando (opcional)</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
+    <row r="11" ht="28" customHeight="1" s="9">
+      <c r="A11" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Hub USB</t>
         </is>
       </c>
-      <c r="C10" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="8" t="inlineStr"/>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="C11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>https://es.aliexpress.com/item/1005009094671557.html?spm=a2g0o.order_list.order_list_main.117.413d194dwWlj7h&amp;gatewayAdapt=glo2esp</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>Sólo para teclado + mando a la vez</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Mando USB</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="6" t="inlineStr"/>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>XInput/Xbox recomendado</t>
-        </is>
-      </c>
-    </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>WiFi (opcional)</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
-      <c r="D12" s="3" t="n"/>
-      <c r="E12" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="13" t="n"/>
+    </row>
+    <row r="13" ht="28" customHeight="1" s="9">
+      <c r="A13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Módulo ESP-01S (ESP8266)</t>
         </is>
       </c>
-      <c r="C13" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="8" t="inlineStr"/>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="C13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>https://es.aliexpress.com/item/1005007199950424.html?spm=a2g0o.productlist.main.4.46e91e1eCw0NXy&amp;aem_p4p_detail=202605310955163358756173391200003156850&amp;algo_pvid=59baa91a-1bd4-4c3d-abc4-da3f9fa92604&amp;algo_exp_id=59baa91a-1bd4-4c3d-abc4-da3f9fa92604-3&amp;pdp_ext_f=%7B%22order%22%3A%22115%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%217.69%217.69%21%21%2159.20%2159.20%21%40211b6c1917802465165527071e666a%2112000039781880873%21sea%21ES%21129485342%21X%211%210%21n_tag%3A-29919%3Bd%3A90000c2b%3Bm03_new_user%3A-29895&amp;curPageLogUid=fEYHOSyp5NIc&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005007199950424%7C_p_origin_prod%3A&amp;search_p4p_id=202605310955163358756173391200003156850_1</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>TX→pin 77, RX→pin 73, VCC→3.3V, GND→GND · firmware ducasp ESPFW1.4 (OCM)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Cables / jumpers para ESP</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="6" t="inlineStr"/>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>Conexión al header GPIO</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>Carcasa</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Carcasa impresa en 3D (PETG blanco)</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="8" t="inlineStr"/>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>STL/3MF en case/ · ver hoja "Piezas 3D (case)"</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Tornillería / separadores</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="6" t="inlineStr"/>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>según carcasa (rellenar)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="3">
+    <mergeCell ref="A1:E1"/>
     <mergeCell ref="A12:E12"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A9:E9"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>